<commit_message>
Final build-verification wrap-up docs across all three projects (2026-08-19)
- Refresh BUILD-VERIFICATION-COVERAGE: all three projects build-verified
  (RS 437/71/508, Schedule 190/5/195 incl. Stefan-deploy re-check + Priority fix,
  Filters 119/5/124); grand total 746/81/827. The one staging item left = the
  PV CSV rule + WIP Story-5 reconciliation (~15 cases), blocked on fresh cookies.
- Regenerate both Defects-for-Testers .xlsx to match their annotated .md twins
  (0 mismatches; RS 35 rows, Schedule 2+2+7).
- Refresh SPOT-CHECK-SAMPLE: add Schedule (5) + Filters (6) nominees -> 44 C-ids.
- Add EXECUTIVE-SUMMARY-2026-08-19 (one-page action-first status).
- Update OUTSTANDING-ITEMS-REGISTER final consolidated state.

Docs-only; no staging/TestRail/Jira/test-case writes.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/report-suite/build-verify-2026-08-18/Defects-for-Testers_ReportSuite-and-Schedule_2026-08-19.xlsx
+++ b/build/report-suite/build-verify-2026-08-18/Defects-for-Testers_ReportSuite-and-Schedule_2026-08-19.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,22 +32,11 @@
       <sz val="13"/>
     </font>
     <font>
-      <i val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -66,7 +55,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -74,11 +63,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -86,21 +89,15 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -466,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A1:L80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -478,135 +475,401 @@
     <col width="34" customWidth="1" min="7" max="7"/>
     <col width="30" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
     <col width="34" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Defects for Manual Testers — Report Suite &amp; Schedule (build v3.8-bd246fd) — 2026-08-19</t>
+          <t>Defects for Manual Testers — Report Suite &amp; Schedule (2026-08-19)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Jira ticket creation is ON HOLD; this is a read-only file for the manual testers to review. Expected behavior comes from the documented source (spec / epic / PO answer), never the build (Standing Rule 57).</t>
+          <t>Build: v3.8-bd246fd. Jira ticket creation is ON HOLD — this is a read-only file for the manual testers to review.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>UPDATE 2026-08-19 (1st message) — Chris Ward answered the WIP PO questions. Row 28 (WIP tab-placement self-contradiction) is RESOLVED — he tidied the live spec to the line-state model (new S3-R5/S3-R6). A pending-Chris item, row 35 (WIP per-line aging), was added.</t>
+          <t>Expected behavior comes from the documented source (spec / epic / PO answer), never the build (Standing Rule 57).</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>UPDATE 2026-08-19 (2nd message) — row 35 is now RESOLVED too. Chris ruled aging is per job and "that's final"; the shared Days Open value on a two-row job is CORRECT (not a bug); the stray per-line line is gone as of spec page v24. A separate Quote Age column is future work — SV-9372 (Parth, not started); nothing to test — do NOT file the shared Days Open value as a defect in the meantime.</t>
+          <t>UPDATE 2026-08-19 (1st message) — Chris Ward answered the WIP PO questions. Row 28 (WIP tab-placement self-contradiction) is RESOLVED — he tidied the live spec to the line-state model (new S3-R5/S3-R6). A pending-Chris item, row 35 (WIP per-line aging), was added.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Schedule batches B (66 cases) and C (68 cases) are PENDING — their defect verdicts cannot be produced until fresh staging cookies land. This file covers Report Suite (all 6 reports) + Schedule batch A only.</t>
+          <t>UPDATE 2026-08-19 (2nd message) — row 35 is now RESOLVED too. Chris ruled aging is per job and *"that's final"*; the shared Days Open value on a two-row job is CORRECT (not a bug); the stray per-line line is gone as of spec page v24. A separate Quote Age column is future work — SV-9372 (Parth, not started); nothing to test — do NOT file the shared Days Open value as a defect in the meantime. Source: build/report-suite/chris-answers-2026-08-19/WIP-CHRIS-RULINGS-2026-08-19.md. ⚠️ The .xlsx twin of this file needs REGENERATION to match these annotations — do not hand-edit the binary.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Schedule batches B (66 cases) and C (68 cases) are PENDING — their defect verdicts cannot be produced until fresh staging cookies land (container reset ~06:30 UTC 2026-08-19 wiped the live session). Any Schedule scheduling-core / events / permissions defects will be added once batches B+C run. This file covers Report Suite (all 6 reports) + Schedule batch A only.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>| # | Project | Report/Area | Title | Description | Steps to Reproduce | Expected behavior | Source | Ticket (key + status) | Reproduces on v3.8-bd246fd? | Affected TestRail case(s) (C-id + link) | Recommendation |</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>|---|---|---|---|---|---|---|---|---|---|---|---|</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>| 1 | Report Suite | Sales By Customer / Sales By Representative | Expanded-View PDF prints on A3, not A4 | The Expanded-View PDF exports on A3 paper (1190.55 x 841.89 pts) while the Summary PDF from the same menu is correctly A4 (841.89 x 595.28). | 1. Open Sales By Customer.&lt;br&gt;2. Switch to Expanded View.&lt;br&gt;3. Open the export menu and choose PDF.&lt;br&gt;4. Open the downloaded file and check its paper size (compare with the Summary PDF). | Both PDFs print on A4 landscape (like the Summary PDF). | SBC report specification S15-R5..R8 (A4 landscape); epic SV-8582. | SV-8964 (OBSOLETE); SBR cross-ref SV-8981 | Yes (pdfinfo on both live downloads) | C30166 (https://shopview.testrail.io/index.php?/cases/view/30166), C30279 (https://shopview.testrail.io/index.php?/cases/view/30279) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>| 2 | Report Suite | Sales By Customer | Chosen date range not saved into the page link | After selecting a date range and clicking Apply, the address bar stays at the plain report URL — the range is not written into the shareable link. | 1. Open Sales By Customer.&lt;br&gt;2. Pick a date range.&lt;br&gt;3. Click Apply.&lt;br&gt;4. Look at the browser address bar. | The chosen date range is written into the page link so re-opening the link restores the same range. | SBC report specification — shareable-link requirement (date range persisted in the URL); epic SV-8582. | SV-8955 (OBSOLETE) | Yes | C30105 (https://shopview.testrail.io/index.php?/cases/view/30105) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>| 3 | Report Suite | Sales By Representative | Empty-state message wording is wrong | The empty-state message reads "No sales data found for the selected filters." — not the spec's standard empty-state wording. | 1. Open Sales By Representative.&lt;br&gt;2. Keep the default (assigned-reps-only) view, which returns no rows.&lt;br&gt;3. Read the empty-state message. | The empty-state shows the spec's standard wording (different from the current text). | SBR report specification — empty-state message wording; epic SV-8582. | SV-8973 (OBSOLETE / Done) | Yes | C30298 (https://shopview.testrail.io/index.php?/cases/view/30298) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>| 4 | Report Suite | Sales By Representative | Icon-button accessible names are wrong | Export three-dot button's accessible name is "Export report" and the column button's is "Column Selection". | 1. Open Sales By Representative.&lt;br&gt;2. With a screen reader or dev tools, read the accessible name of the three-dot export button and of the column button. | Export button = "Report actions"; column button = "Show/Hide columns". | SBR report specification — icon-button accessible names; epic SV-8582. | SV-8975 (OBSOLETE / Done) | Yes | C30307 (https://shopview.testrail.io/index.php?/cases/view/30307) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>| 5 | Report Suite | Parts Velocity | Location filter defaults to All locations | The Location filter opens on "All locations" instead of the user's active location. | 1. Sign in as a user with more than one location.&lt;br&gt;2. Open Parts Velocity.&lt;br&gt;3. Look at the Location filter's default value. | The Location filter defaults to the user's active location, not "All locations". | PV report specification S2-R9 / Chris Ward's decision; epic SV-8582. | SV-8939 (OBSOLETE) | Yes | C30337 (https://shopview.testrail.io/index.php?/cases/view/30337) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>| 6 | Report Suite | Parts Velocity | Long cells not truncated / no hover tooltip | Long Description/Category/Vendor cells are not truncated (computed text-overflow: clip) and have no hover tooltip. | 1. Open Parts Velocity.&lt;br&gt;2. Find a row with a long Description, Category or Vendor value.&lt;br&gt;3. Hover over that cell. | Long text is truncated with an ellipsis and a hover tooltip shows the full value. | PV report specification S3-R7; epic SV-8582. | SV-8940 (OBSOLETE) | Yes | C30347 (https://shopview.testrail.io/index.php?/cases/view/30347) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>| 7 | Report Suite | Parts Velocity | Export success toast is generic | The export success toast reads "Data exported successfully." rather than the specified report-specific wording. | 1. Open Parts Velocity.&lt;br&gt;2. Export CSV (then repeat for PDF).&lt;br&gt;3. Read the success toast. | Toast reads "Velocity report exported (CSV)" / "Velocity report exported (PDF)". | PV report specification S6-R9 / N1; epic SV-8582. | SV-8936 (OBSOLETE) | Yes | C30384 (https://shopview.testrail.io/index.php?/cases/view/30384) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>| 8 | Report Suite | Technician Utilization | Report opens on All locations | The report opens on "All locations", not the user's active shop. | 1. Sign in as a user with more than one location.&lt;br&gt;2. Open Technician Utilization.&lt;br&gt;3. Look at the Location default. | The report opens on the user's active shop. | TU report specification v9 — active-location default; epic SV-8582. | SV-8943 (OBSOLETE) | Yes | C30394 (https://shopview.testrail.io/index.php?/cases/view/30394) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>| 9 | Report Suite | Technician Utilization | Sort/filter fire a server request | Both a column-header sort and a technician-filter deselect fire a server request; the spec requires both to be client-side only. | 1. Open Technician Utilization.&lt;br&gt;2. Open dev tools Network.&lt;br&gt;3. Click a column header to sort.&lt;br&gt;4. Deselect a technician.&lt;br&gt;5. Watch for a server request. | No server request — header sort and technician-filter deselect operate client-side only. | TU report specification v9 — client-side sort/filter; epic SV-8582. | SV-8945 (OBSOLETE) | Yes | C30450 (https://shopview.testrail.io/index.php?/cases/view/30450) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>| 10 | Report Suite | Technician Utilization | Summary row missing from PDF exports | The Summary row is absent from both the Summary PDF and the Expanded PDF (the filename half is fixed). | 1. Open Technician Utilization.&lt;br&gt;2. Export the Summary PDF and the Expanded PDF.&lt;br&gt;3. Look for the Summary row in each file. | The Summary row is present in the PDF exports. | TU report specification v9 — Summary row in exports; epic SV-8582. | SV-8950 (OBSOLETE) | Yes (partial — filename half fixed) | C30435 (https://shopview.testrail.io/index.php?/cases/view/30435) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>| 11 | Report Suite | Technician Utilization | Two CSVs, per-day rows, no Summary row | There are two spreadsheet files, and the Expanded CSV holds a row per day; neither CSV contains the Summary row. | 1. Open Technician Utilization.&lt;br&gt;2. Export the spreadsheet.&lt;br&gt;3. Open the downloaded file(s). | One summary-level technician-utilization.csv containing the Summary row. | TU report specification v9 — single summary-level CSV; epic SV-8582. | SV-8951 (OBSOLETE) | Yes | C30436 (https://shopview.testrail.io/index.php?/cases/view/30436), C43552 (https://shopview.testrail.io/index.php?/cases/view/43552) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>| 12 | Report Suite | Technician Utilization | Export toast wording is wrong | Success toast reads "Data exported successfully."; the failure toast reads "Empty export…". | 1. Open Technician Utilization.&lt;br&gt;2. Start an export and read the success toast.&lt;br&gt;3. Trigger a failing export and read the failure toast. | Success toast = "Download started"; failure toast = "Failed to download report". | TU report specification v9 — export toast wording; epic SV-8582. | SV-8952 (OBSOLETE) | Yes | C30441 (https://shopview.testrail.io/index.php?/cases/view/30441) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>| 13 | Report Suite | Technician Utilization | Location column 2nd, not leftmost, and not in selector | For a multi-location user the Location column is 2nd (after Technician), not leftmost, and Location is never offered in Column Selection. | 1. Sign in as a multi-location user.&lt;br&gt;2. Open Technician Utilization.&lt;br&gt;3. Note the Location column position.&lt;br&gt;4. Open Column Selection and look for Location. | Location column is leftmost (before Technician) and is offered in Column Selection. | TU report specification v9 — Location column position + selector; epic SV-8582. | SV-8954 (OBSOLETE); WIP cross-ref C38916 | Yes | C38915 (https://shopview.testrail.io/index.php?/cases/view/38915) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>| 14 | Report Suite | Technician Utilization | Select-all control labelled "All technicians" | The select-all control is labelled "All technicians", not "Select all" (the behaviour itself passes). | 1. Open Technician Utilization.&lt;br&gt;2. Open the technician multi-select.&lt;br&gt;3. Read the select-all control's label. | The select-all control is labelled "Select all". | TU report specification v9 — select-all label; epic SV-8582. | SV-8947 (OBSOLETE) | Yes (label only) | C30425 (https://shopview.testrail.io/index.php?/cases/view/30425) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>| 15 | Report Suite | Technician Utilization | aria-expanded not reported on expand controls | The expand / expand-all controls have accessible names and keyboard toggles, but aria-expanded is not reported to assistive tech. | 1. Open Technician Utilization.&lt;br&gt;2. Focus a row's expand control (and the expand-all control).&lt;br&gt;3. Inspect the aria-expanded attribute as you toggle. | aria-expanded state is exposed to assistive technology. | TU report specification v9 — accessibility (aria-expanded); epic SV-8582. | SV-8953 (OBSOLETE) | Yes | C30418 (https://shopview.testrail.io/index.php?/cases/view/30418), C30421 (https://shopview.testrail.io/index.php?/cases/view/30421) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>| 16 | Report Suite | Work In Progress | WO # is plain text, no link | WO # is a plain span (black text, no anchor); the whole table has 0 links even for a user WITH Work Orders access. | 1. Sign in as a user WITH Work Orders access.&lt;br&gt;2. Open Work In Progress.&lt;br&gt;3. Try to click a WO # cell. | WO # is a link that opens the work order (for entitled users). | WIP report specification — WO # link for entitled users; epic SV-8582. | SV-8967 (OBSOLETE) | Yes | C30468 (https://shopview.testrail.io/index.php?/cases/view/30468), C43557 (https://shopview.testrail.io/index.php?/cases/view/43557), C30523 (https://shopview.testrail.io/index.php?/cases/view/30523) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>| 17 | Report Suite | Work In Progress | Rows are pale blue-grey, not white | Header, data rows and Totals row are all rgb(249,250,251) (pale blue-grey), not white. | 1. Open Work In Progress.&lt;br&gt;2. Inspect the row background colour. | Rows are white (with no alternating shading). | WIP report specification — row background colour; epic SV-8582. | SV-8970 (OBSOLETE) | Yes (exactly) | C30519 (https://shopview.testrail.io/index.php?/cases/view/30519) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>| 18 | Report Suite | Work In Progress | Numeric column headers/cells left-aligned | Days Open and Last Activity column headers are left-aligned (expected right); the Days Open data cell is also left-aligned. Broader than the ticket named. | 1. Open Work In Progress.&lt;br&gt;2. Check the alignment of the Days Open and Last Activity column headers and the Days Open data cells. | Numeric/right-hand columns (Days Open, Last Activity) are right-aligned. | WIP report specification — column alignment; epic SV-8582. | SV-8987 (OBSOLETE) | Yes (broader than the ticket) | C30466 (https://shopview.testrail.io/index.php?/cases/view/30466) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>| 19 | Report Suite | Work In Progress | Estimates summary figure not muted | The Estimates summary figure is rgb(54,65,82) — identical to the others — so it is not toned down/muted. | 1. Open Work In Progress.&lt;br&gt;2. Compare the colour of the Estimates summary figure to the Completed and Not-Started figures. | The Estimates summary figure is toned down / muted relative to the others. | WIP report specification — Estimates summary styling; epic SV-8582. | SV-8988 (OBSOLETE) | Yes | C30491 (https://shopview.testrail.io/index.php?/cases/view/30491) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>| 20 | Report Suite | Work In Progress | Labor Delta shows two decimals | Labor Delta shows two decimals (+3.00, +2.20); expected one decimal. Sign is correct. | 1. Open Work In Progress.&lt;br&gt;2. Read a Labor Delta value. | Labor Delta shows one decimal (e.g. +3.0). | WIP report specification — Labor Delta formatting; epic SV-8582. | SV-8989 (OBSOLETE) | Yes | C30481 (https://shopview.testrail.io/index.php?/cases/view/30481) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>| 21 | Report Suite | Work In Progress | Customer filter offers Clear before any selection | The Customer filter shows "Clear all" before anything is selected. | 1. Open Work In Progress.&lt;br&gt;2. Open the Customer filter without selecting anything.&lt;br&gt;3. Look for a Clear action. | No Clear action until at least one selection is made; then it is labelled "Clear". | WIP report specification — filter Clear behaviour; epic SV-8582. | SV-8969 (OBSOLETE) | Yes | C30499 (https://shopview.testrail.io/index.php?/cases/view/30499) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>| 22 | Report Suite | Work In Progress | Filter change fires a server request | Changing a filter (e.g. Advisor) fires one server request (server-side recompute); figures are correct either way. | 1. Open Work In Progress.&lt;br&gt;2. Open dev tools Network.&lt;br&gt;3. Change a filter (e.g. Advisor).&lt;br&gt;4. Watch for a server request. | The filter narrows the results on-screen with no server request. | WIP report specification — client-side filter narrowing; epic SV-8582. | SV-8968 (OBSOLETE) | Yes | C30505 (https://shopview.testrail.io/index.php?/cases/view/30505), C30498 (https://shopview.testrail.io/index.php?/cases/view/30498) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>| 23 | Report Suite | Inventory Value | Totals row reads "Totals" not "Total" | The Totals row's first cell reads "Totals"; the spec asks for "Total". | 1. Open Inventory Value.&lt;br&gt;2. Read the first cell of the Totals row. | The Totals row's first cell reads "Total". | IV report specification v10 S4-R1; epic SV-8582. | SV-8926 (OBSOLETE) | Yes | C30556 (https://shopview.testrail.io/index.php?/cases/view/30556) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>| 24 | Report Suite | Inventory Value | Empty-state wording differs from spec | The empty-state message reads "No inventory value to show for this selection." — not the spec's standard wording. | 1. Open Inventory Value.&lt;br&gt;2. Apply a selection that returns no rows.&lt;br&gt;3. Read the empty-state message. | The empty-state shows the spec's standard wording: "Empty bays, endless possibilities. Get Going!". | IV report specification v10 — standard empty-state wording; epic SV-8582. | SV-8930 (OBSOLETE) | Yes (different wording) | C30539 (https://shopview.testrail.io/index.php?/cases/view/30539) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>| 25 | Report Suite | Inventory Value | First visit opens All locations | On first visit (fresh browser context) the report opens on "All locations", not the active location. | 1. Open Inventory Value in a fresh browser context.&lt;br&gt;2. Check the Location default. | First visit opens on the user's active location. | IV report specification v10 S1-R3 / S7-R2; epic SV-8582. | SV-8931 (OBSOLETE) | Yes | C30536 (https://shopview.testrail.io/index.php?/cases/view/30536), C30574 (https://shopview.testrail.io/index.php?/cases/view/30574) | REOPEN |</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>| 26 | Report Suite | Technician Utilization | Empty export shows an error toast instead of silent no-op | Exporting with all technicians cleared shows an "Empty export / Export didn't yield any results" error toast, not the spec's silent no-op. Differs from BOTH the spec and the old SV-8948 symptom. | 1. Open Technician Utilization.&lt;br&gt;2. Deselect all technicians.&lt;br&gt;3. Trigger an export. | A silent no-op — no file is produced and no message is shown. | TU report specification v9 S7-N1 (silent no-op); epic SV-8582. | NO TICKET (new deviation) | Yes (new deviation) | C30440 (https://shopview.testrail.io/index.php?/cases/view/30440) | FILE-NEW |</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>| 27 | Report Suite | Sales By Representative / Inventory Value | CSV money now plain numbers (appears fixed) | CSV money is now written as plain numbers, not "$…" text; IV column order is also correct (Total Cost last). | 1. Open Sales By Representative (then Inventory Value).&lt;br&gt;2. Export CSV.&lt;br&gt;3. Open the file and check the money columns (and IV column order). | CSV money is plain numbers; IV Total Cost is the last column. | SBR / IV report specifications — CSV money format + IV column order; epic SV-8582. | SV-8823 (OPEN — TESTING QA) | No — appears FIXED on v3.8 | C30287 (https://shopview.testrail.io/index.php?/cases/view/30287), C30589 (https://shopview.testrail.io/index.php?/cases/view/30589) | CLOSE-AS-FIXED (first verify the CSV honours column-selection-in-export — IV sub-claim not tested; C30588 keeps an SV-8823 note) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>| 28 | Report Suite | Work In Progress | ✅ RESOLVED 2026-08-19 — PO question: WIP tab-placement spec self-contradiction | The spec carried BOTH placement models: S2-R4 ("appears once, in one tab") vs the SV-9027 line-state Key Decision ("appears in each matching tab"). RESOLVED by Chris Ward 2026-08-19 — he tidied the LIVE Confluence spec so Story 3 and S2-R4 now describe the line-state model (new S3-R5, S3-R6). Our cases already follow line-state (his 2026-08-18 answer B), so they now agree with the tidied spec; the divergence note can be retired. Still owed: pull the live page (local baseline v22 is behind). | 1. Open Work In Progress.&lt;br&gt;2. Find a work order with lines in more than one state.&lt;br&gt;3. Note which tab(s) it appears in.&lt;br&gt;(Note: no such WO exists in current data — needs seeding.) | Per the current documents (now consistent): a work order appears in each matching tab by line state (line-state model). | WIP report specification — live Confluence (line-state model, new S3-R5/S3-R6); Chris Ward ruling 2026-08-19. | N/A (document conflict — RESOLVED by PO) | Not established (no multi-state WO in data) | C30456 (https://shopview.testrail.io/index.php?/cases/view/30456), C30458 (https://shopview.testrail.io/index.php?/cases/view/30458), C43979 (https://shopview.testrail.io/index.php?/cases/view/43979) | RESOLVED (Chris Ward 2026-08-19 tidied the live spec to line-state; pull live page — register RS-WIP-6) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>| 29 | Report Suite | Sales By Customer / Sales By Representative | PO question: invoice number — link or plain text? | The build renders the invoice number as a plain-text span (no href), but the spec states BOTH: S9-N2 (link to access-denied) and S9-R1a (plain-text, no link). | 1. Open Sales By Customer (and Sales By Representative).&lt;br&gt;2. Look at an invoice number cell — is it a link or plain text? | Per the intended (to-be-confirmed) document: whichever of link / plain-text Chris Ward confirms. | SBC / SBR report specifications — conflict between S9-N2 and S9-R1a. | N/A (document conflict — not a defect) | N/A (build shows plain text; conflict unresolved) | C30100 (https://shopview.testrail.io/index.php?/cases/view/30100), C43558 (https://shopview.testrail.io/index.php?/cases/view/43558), C30138 (https://shopview.testrail.io/index.php?/cases/view/30138) | PO-QUESTION (chase Chris Ward for the intended behaviour) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>| 30 | Report Suite | Parts Velocity | PO question: Location column position | SV-8938 says the Location column should be leftmost (before Type), but the spec says two different things (S3-R10 access-gated/toggleable vs S2-R12 scope-tied), and the 20 picker columns don't list Location. The column sits 6th on screen and in CSV. | 1. Sign in as a multi-location user.&lt;br&gt;2. Open Parts Velocity.&lt;br&gt;3. Note the Location column position on screen and in the CSV export. | Per the intended (to-be-confirmed) document: the position/toggle behaviour Chris Ward confirms. | PV report specification — conflict between S3-R10 and S2-R12; contested ticket SV-8938. | SV-8938 (contested) | Column sits 6th (on screen + CSV); "leftmost" not confirmed | C38914 (https://shopview.testrail.io/index.php?/cases/view/38914), C30352 (https://shopview.testrail.io/index.php?/cases/view/30352) | PO-QUESTION (get Chris Ward's answer before reopening/refiling SV-8938) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>| 31 | Report Suite | Parts Velocity | PDF export fails (SV-8818) | PDF export returns HTTP 500 on a medium view while CSV works; over-cap views are correctly refused with the standard message. | 1. Open Parts Velocity.&lt;br&gt;2. Load a medium-sized view.&lt;br&gt;3. Export PDF. | PDF export returns a downloadable file (HTTP 200). | PV report specification — PDF export requirement; epic SV-8582. | SV-8818 (OPEN — TESTING QA) | Yes (PDF 500) | C38885 (https://shopview.testrail.io/index.php?/cases/view/38885), C43547 (https://shopview.testrail.io/index.php?/cases/view/43547) | KEEP-EXPECT-FAIL |</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>| 32 | Report Suite | Inventory Value | PDF export fails on large view (SV-8818) | PDF export times out / returns 500 on the large IV view (5,703 rows); small filtered views work (HTTP 200). | 1. Open Inventory Value.&lt;br&gt;2. Load the large (all-locations) view.&lt;br&gt;3. Export PDF. | PDF export returns a downloadable file (HTTP 200). | IV report specification v10 — PDF export requirement; epic SV-8582. | SV-8818 (OPEN — TESTING QA) | Yes (PDF 500/timeout on large view) | C30587 (https://shopview.testrail.io/index.php?/cases/view/30587), C30590 (https://shopview.testrail.io/index.php?/cases/view/30590), C30591 (https://shopview.testrail.io/index.php?/cases/view/30591), C30593 (https://shopview.testrail.io/index.php?/cases/view/30593), C30595 (https://shopview.testrail.io/index.php?/cases/view/30595), C43548 (https://shopview.testrail.io/index.php?/cases/view/43548) | KEEP-EXPECT-FAIL |</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>| 33 | Report Suite | Sales By Representative | Over-cap Expanded PDF / API row-cap (SV-8818) | The &gt; row-cap Expanded-PDF / API state is not reachable at 88 invoices; base exports return 200. Kept EXPECT-FAIL pending a seedable over-cap state. | 1. Open Sales By Representative.&lt;br&gt;2. Build a view that exceeds the row cap (not reachable at 88 invoices — needs seeding).&lt;br&gt;3. Export the Expanded PDF. | Over-cap export is refused with the standard row-cap message. | SBR report specification — export row-cap; epic SV-8582. | SV-8818 (OPEN — TESTING QA) | Not reachable at 88 invoices (base exports 200) | C30290 (https://shopview.testrail.io/index.php?/cases/view/30290), C30320 (https://shopview.testrail.io/index.php?/cases/view/30320) | KEEP-EXPECT-FAIL |</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>| 34 | Schedule | Sidebar - Work Order Filters | Priority filter group missing from the sidebar Filters panel | The sidebar Filters popup contains only Assignment (Unassigned/Assigned) and Status; there is no Priority group (High/Medium/Low). Confirmed by reading the full popup and a body-wide search. | 1. Open Schedule.&lt;br&gt;2. Click the sidebar Filters button.&lt;br&gt;3. Look for a Priority group with High / Medium / Low options. | The Filters panel offers three groups: Assignment, Status, and Priority (High, Medium, Low). | Schedule specification v30 §5.1 / story SV-8687; epic SV-8685. | NO TICKET (feature not found — Rule 69 deferred) | Yes (Priority group absent on v3.8-bd246fd) | C29945 (https://shopview.testrail.io/index.php?/cases/view/29945) | DEFERRED (feature not found — confirm with Branko whether Priority filtering is in V1; re-check when it ships) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>| 35 | Report Suite | Work In Progress | ✅ RESOLVED 2026-08-19 — WIP aging is per job (FINAL); shared Days Open on a two-row job is correct | Chris Ward's 2nd message ruled aging is per job, and *"that's final"*. Days Open is whole days since the work order's date; a two-row job (status tab + Estimates) shows the same number on both rows — *"the money splits by line state, the clock doesn't"* — and that shared number is CORRECT behaviour, not a bug. The stray per-line-aging line is gone from the spec as of page v24, so nothing conflicts. A separate Quote Age column is future work — SV-9372 (Parth, not started); nothing to test — do NOT file the shared Days Open value as a defect in the meantime. | 1. Open Work In Progress.&lt;br&gt;2. Read the Days Open value for a work order that has both approved and unapproved lines (and appears on two tabs).&lt;br&gt;3. Confirm it counts whole days since the work order's date (not per line), and that both rows show the same number. | Days Open = whole days since the work order's date (S4-R12), per job; both rows of a two-row job show the same number (correct, not a defect). Per-line aging is NOT built — do not test for it. A future Quote Age column (SV-9372) is not yet built — nothing to test. | WIP report specification S4-R12 (per-line line removed as of page v24); Chris Ward 2nd ruling 2026-08-19. | N/A (RESOLVED by PO — per job, final) | Whole-job Days Open builds correctly; shared value on a two-row job is correct | C30472 (https://shopview.testrail.io/index.php?/cases/view/30472) | RESOLVED (Chris Ward 2026-08-19 — aging per job, final; do NOT file the shared Days Open value as a defect; SV-9372 Quote Age is future — register RS-WIP-4 cleared, RS-WIP-7 opened) |</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>Report/Area</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E45" s="3" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>Steps to Reproduce</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G45" s="3" t="inlineStr">
         <is>
           <t>Expected behavior</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H45" s="3" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I45" s="3" t="inlineStr">
         <is>
           <t>Ticket (key + status)</t>
         </is>
       </c>
-      <c r="J7" s="3" t="inlineStr">
+      <c r="J45" s="3" t="inlineStr">
         <is>
           <t>Reproduces on v3.8-bd246fd?</t>
         </is>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K45" s="3" t="inlineStr">
         <is>
           <t>Affected TestRail case(s) (C-id + link)</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="L45" s="3" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>Sales By Customer / Sales By Representative</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D46" s="4" t="inlineStr">
         <is>
           <t>Expanded-View PDF prints on A3, not A4</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E46" s="4" t="inlineStr">
         <is>
           <t>The Expanded-View PDF exports on A3 paper (1190.55 x 841.89 pts) while the Summary PDF from the same menu is correctly A4 (841.89 x 595.28).</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F46" s="4" t="inlineStr">
         <is>
           <t>1. Open Sales By Customer.
 2. Switch to Expanded View.
@@ -614,64 +877,64 @@
 4. Open the downloaded file and check its paper size (compare with the Summary PDF).</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G46" s="4" t="inlineStr">
         <is>
           <t>Both PDFs print on A4 landscape (like the Summary PDF).</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H46" s="4" t="inlineStr">
         <is>
           <t>SBC report specification S15-R5..R8 (A4 landscape); epic SV-8582.</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I46" s="4" t="inlineStr">
         <is>
           <t>SV-8964 (OBSOLETE); SBR cross-ref SV-8981</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J46" s="4" t="inlineStr">
         <is>
           <t>Yes (pdfinfo on both live downloads)</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K46" s="4" t="inlineStr">
         <is>
           <t>C30166 (https://shopview.testrail.io/index.php?/cases/view/30166), C30279 (https://shopview.testrail.io/index.php?/cases/view/30279)</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L46" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>Sales By Customer</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D47" s="4" t="inlineStr">
         <is>
           <t>Chosen date range not saved into the page link</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E47" s="4" t="inlineStr">
         <is>
           <t>After selecting a date range and clicking Apply, the address bar stays at the plain report URL — the range is not written into the shareable link.</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F47" s="4" t="inlineStr">
         <is>
           <t>1. Open Sales By Customer.
 2. Pick a date range.
@@ -679,447 +942,447 @@
 4. Look at the browser address bar.</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G47" s="4" t="inlineStr">
         <is>
           <t>The chosen date range is written into the page link so re-opening the link restores the same range.</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H47" s="4" t="inlineStr">
         <is>
           <t>SBC report specification — shareable-link requirement (date range persisted in the URL); epic SV-8582.</t>
         </is>
       </c>
-      <c r="I9" s="4" t="inlineStr">
+      <c r="I47" s="4" t="inlineStr">
         <is>
           <t>SV-8955 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J9" s="4" t="inlineStr">
+      <c r="J47" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K9" s="4" t="inlineStr">
+      <c r="K47" s="4" t="inlineStr">
         <is>
           <t>C30105 (https://shopview.testrail.io/index.php?/cases/view/30105)</t>
         </is>
       </c>
-      <c r="L9" s="4" t="inlineStr">
+      <c r="L47" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>Sales By Representative</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D48" s="4" t="inlineStr">
         <is>
           <t>Empty-state message wording is wrong</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>The empty-state message reads "No sales data found for the selected filters." — not the spec's standard empty-state wording.</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F48" s="4" t="inlineStr">
         <is>
           <t>1. Open Sales By Representative.
 2. Keep the default (assigned-reps-only) view, which returns no rows.
 3. Read the empty-state message.</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>The empty-state shows the spec's standard wording (different from the current text).</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>SBR report specification — empty-state message wording; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I10" s="4" t="inlineStr">
+      <c r="I48" s="4" t="inlineStr">
         <is>
           <t>SV-8973 (OBSOLETE / Done)</t>
         </is>
       </c>
-      <c r="J10" s="4" t="inlineStr">
+      <c r="J48" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K10" s="4" t="inlineStr">
+      <c r="K48" s="4" t="inlineStr">
         <is>
           <t>C30298 (https://shopview.testrail.io/index.php?/cases/view/30298)</t>
         </is>
       </c>
-      <c r="L10" s="4" t="inlineStr">
+      <c r="L48" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>Sales By Representative</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Icon-button accessible names are wrong</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>Export three-dot button's accessible name is "Export report" and the column button's is "Column Selection".</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F49" s="4" t="inlineStr">
         <is>
           <t>1. Open Sales By Representative.
 2. With a screen reader or dev tools, read the accessible name of the three-dot export button and of the column button.</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G49" s="4" t="inlineStr">
         <is>
           <t>Export button = "Report actions"; column button = "Show/Hide columns".</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H49" s="4" t="inlineStr">
         <is>
           <t>SBR report specification — icon-button accessible names; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="I49" s="4" t="inlineStr">
         <is>
           <t>SV-8975 (OBSOLETE / Done)</t>
         </is>
       </c>
-      <c r="J11" s="4" t="inlineStr">
+      <c r="J49" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K11" s="4" t="inlineStr">
+      <c r="K49" s="4" t="inlineStr">
         <is>
           <t>C30307 (https://shopview.testrail.io/index.php?/cases/view/30307)</t>
         </is>
       </c>
-      <c r="L11" s="4" t="inlineStr">
+      <c r="L49" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>Parts Velocity</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>Location filter defaults to All locations</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E50" s="4" t="inlineStr">
         <is>
           <t>The Location filter opens on "All locations" instead of the user's active location.</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F50" s="4" t="inlineStr">
         <is>
           <t>1. Sign in as a user with more than one location.
 2. Open Parts Velocity.
 3. Look at the Location filter's default value.</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G50" s="4" t="inlineStr">
         <is>
           <t>The Location filter defaults to the user's active location, not "All locations".</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>PV report specification S2-R9 / Chris Ward's decision; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
+      <c r="I50" s="4" t="inlineStr">
         <is>
           <t>SV-8939 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J12" s="4" t="inlineStr">
+      <c r="J50" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K12" s="4" t="inlineStr">
+      <c r="K50" s="4" t="inlineStr">
         <is>
           <t>C30337 (https://shopview.testrail.io/index.php?/cases/view/30337)</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L50" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>Parts Velocity</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>Long cells not truncated / no hover tooltip</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E51" s="4" t="inlineStr">
         <is>
           <t>Long Description/Category/Vendor cells are not truncated (computed text-overflow: clip) and have no hover tooltip.</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F51" s="4" t="inlineStr">
         <is>
           <t>1. Open Parts Velocity.
 2. Find a row with a long Description, Category or Vendor value.
 3. Hover over that cell.</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G51" s="4" t="inlineStr">
         <is>
           <t>Long text is truncated with an ellipsis and a hover tooltip shows the full value.</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H51" s="4" t="inlineStr">
         <is>
           <t>PV report specification S3-R7; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I13" s="4" t="inlineStr">
+      <c r="I51" s="4" t="inlineStr">
         <is>
           <t>SV-8940 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J13" s="4" t="inlineStr">
+      <c r="J51" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K13" s="4" t="inlineStr">
+      <c r="K51" s="4" t="inlineStr">
         <is>
           <t>C30347 (https://shopview.testrail.io/index.php?/cases/view/30347)</t>
         </is>
       </c>
-      <c r="L13" s="4" t="inlineStr">
+      <c r="L51" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
         <is>
           <t>Parts Velocity</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D52" s="4" t="inlineStr">
         <is>
           <t>Export success toast is generic</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E52" s="4" t="inlineStr">
         <is>
           <t>The export success toast reads "Data exported successfully." rather than the specified report-specific wording.</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F52" s="4" t="inlineStr">
         <is>
           <t>1. Open Parts Velocity.
 2. Export CSV (then repeat for PDF).
 3. Read the success toast.</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G52" s="4" t="inlineStr">
         <is>
           <t>Toast reads "Velocity report exported (CSV)" / "Velocity report exported (PDF)".</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>PV report specification S6-R9 / N1; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="I52" s="4" t="inlineStr">
         <is>
           <t>SV-8936 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J14" s="4" t="inlineStr">
+      <c r="J52" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K14" s="4" t="inlineStr">
+      <c r="K52" s="4" t="inlineStr">
         <is>
           <t>C30384 (https://shopview.testrail.io/index.php?/cases/view/30384)</t>
         </is>
       </c>
-      <c r="L14" s="4" t="inlineStr">
+      <c r="L52" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D53" s="4" t="inlineStr">
         <is>
           <t>Report opens on All locations</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E53" s="4" t="inlineStr">
         <is>
           <t>The report opens on "All locations", not the user's active shop.</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F53" s="4" t="inlineStr">
         <is>
           <t>1. Sign in as a user with more than one location.
 2. Open Technician Utilization.
 3. Look at the Location default.</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G53" s="4" t="inlineStr">
         <is>
           <t>The report opens on the user's active shop.</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H53" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — active-location default; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I15" s="4" t="inlineStr">
+      <c r="I53" s="4" t="inlineStr">
         <is>
           <t>SV-8943 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J15" s="4" t="inlineStr">
+      <c r="J53" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K15" s="4" t="inlineStr">
+      <c r="K53" s="4" t="inlineStr">
         <is>
           <t>C30394 (https://shopview.testrail.io/index.php?/cases/view/30394)</t>
         </is>
       </c>
-      <c r="L15" s="4" t="inlineStr">
+      <c r="L53" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="4" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
         <is>
           <t>9</t>
         </is>
       </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C54" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D54" s="4" t="inlineStr">
         <is>
           <t>Sort/filter fire a server request</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E54" s="4" t="inlineStr">
         <is>
           <t>Both a column-header sort and a technician-filter deselect fire a server request; the spec requires both to be client-side only.</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F54" s="4" t="inlineStr">
         <is>
           <t>1. Open Technician Utilization.
 2. Open dev tools Network.
@@ -1128,256 +1391,256 @@
 5. Watch for a server request.</t>
         </is>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="G54" s="4" t="inlineStr">
         <is>
           <t>No server request — header sort and technician-filter deselect operate client-side only.</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — client-side sort/filter; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I16" s="4" t="inlineStr">
+      <c r="I54" s="4" t="inlineStr">
         <is>
           <t>SV-8945 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J16" s="4" t="inlineStr">
+      <c r="J54" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K16" s="4" t="inlineStr">
+      <c r="K54" s="4" t="inlineStr">
         <is>
           <t>C30450 (https://shopview.testrail.io/index.php?/cases/view/30450)</t>
         </is>
       </c>
-      <c r="L16" s="4" t="inlineStr">
+      <c r="L54" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="4" t="inlineStr">
         <is>
           <t>10</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D55" s="4" t="inlineStr">
         <is>
           <t>Summary row missing from PDF exports</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E55" s="4" t="inlineStr">
         <is>
           <t>The Summary row is absent from both the Summary PDF and the Expanded PDF (the filename half is fixed).</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F55" s="4" t="inlineStr">
         <is>
           <t>1. Open Technician Utilization.
 2. Export the Summary PDF and the Expanded PDF.
 3. Look for the Summary row in each file.</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G55" s="4" t="inlineStr">
         <is>
           <t>The Summary row is present in the PDF exports.</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H55" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — Summary row in exports; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I17" s="4" t="inlineStr">
+      <c r="I55" s="4" t="inlineStr">
         <is>
           <t>SV-8950 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J55" s="4" t="inlineStr">
         <is>
           <t>Yes (partial — filename half fixed)</t>
         </is>
       </c>
-      <c r="K17" s="4" t="inlineStr">
+      <c r="K55" s="4" t="inlineStr">
         <is>
           <t>C30435 (https://shopview.testrail.io/index.php?/cases/view/30435)</t>
         </is>
       </c>
-      <c r="L17" s="4" t="inlineStr">
+      <c r="L55" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
         <is>
           <t>11</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C56" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D56" s="4" t="inlineStr">
         <is>
           <t>Two CSVs, per-day rows, no Summary row</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E56" s="4" t="inlineStr">
         <is>
           <t>There are two spreadsheet files, and the Expanded CSV holds a row per day; neither CSV contains the Summary row.</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F56" s="4" t="inlineStr">
         <is>
           <t>1. Open Technician Utilization.
 2. Export the spreadsheet.
 3. Open the downloaded file(s).</t>
         </is>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>One summary-level technician-utilization.csv containing the Summary row.</t>
         </is>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H56" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — single summary-level CSV; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I18" s="4" t="inlineStr">
+      <c r="I56" s="4" t="inlineStr">
         <is>
           <t>SV-8951 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J18" s="4" t="inlineStr">
+      <c r="J56" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K18" s="4" t="inlineStr">
+      <c r="K56" s="4" t="inlineStr">
         <is>
           <t>C30436 (https://shopview.testrail.io/index.php?/cases/view/30436), C43552 (https://shopview.testrail.io/index.php?/cases/view/43552)</t>
         </is>
       </c>
-      <c r="L18" s="4" t="inlineStr">
+      <c r="L56" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="4" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
         <is>
           <t>12</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="B57" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D57" s="4" t="inlineStr">
         <is>
           <t>Export toast wording is wrong</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E57" s="4" t="inlineStr">
         <is>
           <t>Success toast reads "Data exported successfully."; the failure toast reads "Empty export…".</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr">
+      <c r="F57" s="4" t="inlineStr">
         <is>
           <t>1. Open Technician Utilization.
 2. Start an export and read the success toast.
 3. Trigger a failing export and read the failure toast.</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G57" s="4" t="inlineStr">
         <is>
           <t>Success toast = "Download started"; failure toast = "Failed to download report".</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H57" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — export toast wording; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I19" s="4" t="inlineStr">
+      <c r="I57" s="4" t="inlineStr">
         <is>
           <t>SV-8952 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J19" s="4" t="inlineStr">
+      <c r="J57" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K19" s="4" t="inlineStr">
+      <c r="K57" s="4" t="inlineStr">
         <is>
           <t>C30441 (https://shopview.testrail.io/index.php?/cases/view/30441)</t>
         </is>
       </c>
-      <c r="L19" s="4" t="inlineStr">
+      <c r="L57" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
         <is>
           <t>13</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D58" s="4" t="inlineStr">
         <is>
           <t>Location column 2nd, not leftmost, and not in selector</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E58" s="4" t="inlineStr">
         <is>
           <t>For a multi-location user the Location column is 2nd (after Technician), not leftmost, and Location is never offered in Column Selection.</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="F58" s="4" t="inlineStr">
         <is>
           <t>1. Sign in as a multi-location user.
 2. Open Technician Utilization.
@@ -1385,572 +1648,572 @@
 4. Open Column Selection and look for Location.</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G58" s="4" t="inlineStr">
         <is>
           <t>Location column is leftmost (before Technician) and is offered in Column Selection.</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — Location column position + selector; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="I58" s="4" t="inlineStr">
         <is>
           <t>SV-8954 (OBSOLETE); WIP cross-ref C38916</t>
         </is>
       </c>
-      <c r="J20" s="4" t="inlineStr">
+      <c r="J58" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K20" s="4" t="inlineStr">
+      <c r="K58" s="4" t="inlineStr">
         <is>
           <t>C38915 (https://shopview.testrail.io/index.php?/cases/view/38915)</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L58" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>14</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>Select-all control labelled "All technicians"</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E59" s="4" t="inlineStr">
         <is>
           <t>The select-all control is labelled "All technicians", not "Select all" (the behaviour itself passes).</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr">
+      <c r="F59" s="4" t="inlineStr">
         <is>
           <t>1. Open Technician Utilization.
 2. Open the technician multi-select.
 3. Read the select-all control's label.</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G59" s="4" t="inlineStr">
         <is>
           <t>The select-all control is labelled "Select all".</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H59" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — select-all label; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I21" s="4" t="inlineStr">
+      <c r="I59" s="4" t="inlineStr">
         <is>
           <t>SV-8947 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J21" s="4" t="inlineStr">
+      <c r="J59" s="4" t="inlineStr">
         <is>
           <t>Yes (label only)</t>
         </is>
       </c>
-      <c r="K21" s="4" t="inlineStr">
+      <c r="K59" s="4" t="inlineStr">
         <is>
           <t>C30425 (https://shopview.testrail.io/index.php?/cases/view/30425)</t>
         </is>
       </c>
-      <c r="L21" s="4" t="inlineStr">
+      <c r="L59" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="4" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>15</t>
         </is>
       </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>aria-expanded not reported on expand controls</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E60" s="4" t="inlineStr">
         <is>
           <t>The expand / expand-all controls have accessible names and keyboard toggles, but aria-expanded is not reported to assistive tech.</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="F60" s="4" t="inlineStr">
         <is>
           <t>1. Open Technician Utilization.
 2. Focus a row's expand control (and the expand-all control).
 3. Inspect the aria-expanded attribute as you toggle.</t>
         </is>
       </c>
-      <c r="G22" s="4" t="inlineStr">
+      <c r="G60" s="4" t="inlineStr">
         <is>
           <t>aria-expanded state is exposed to assistive technology.</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 — accessibility (aria-expanded); epic SV-8582.</t>
         </is>
       </c>
-      <c r="I22" s="4" t="inlineStr">
+      <c r="I60" s="4" t="inlineStr">
         <is>
           <t>SV-8953 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J22" s="4" t="inlineStr">
+      <c r="J60" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K22" s="4" t="inlineStr">
+      <c r="K60" s="4" t="inlineStr">
         <is>
           <t>C30418 (https://shopview.testrail.io/index.php?/cases/view/30418), C30421 (https://shopview.testrail.io/index.php?/cases/view/30421)</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L60" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="B23" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t>WO # is plain text, no link</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E61" s="4" t="inlineStr">
         <is>
           <t>WO # is a plain span (black text, no anchor); the whole table has 0 links even for a user WITH Work Orders access.</t>
         </is>
       </c>
-      <c r="F23" s="4" t="inlineStr">
+      <c r="F61" s="4" t="inlineStr">
         <is>
           <t>1. Sign in as a user WITH Work Orders access.
 2. Open Work In Progress.
 3. Try to click a WO # cell.</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G61" s="4" t="inlineStr">
         <is>
           <t>WO # is a link that opens the work order (for entitled users).</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H61" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — WO # link for entitled users; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I23" s="4" t="inlineStr">
+      <c r="I61" s="4" t="inlineStr">
         <is>
           <t>SV-8967 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J23" s="4" t="inlineStr">
+      <c r="J61" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K23" s="4" t="inlineStr">
+      <c r="K61" s="4" t="inlineStr">
         <is>
           <t>C30468 (https://shopview.testrail.io/index.php?/cases/view/30468), C43557 (https://shopview.testrail.io/index.php?/cases/view/43557), C30523 (https://shopview.testrail.io/index.php?/cases/view/30523)</t>
         </is>
       </c>
-      <c r="L23" s="4" t="inlineStr">
+      <c r="L61" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
         <is>
           <t>17</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C62" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D62" s="4" t="inlineStr">
         <is>
           <t>Rows are pale blue-grey, not white</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E62" s="4" t="inlineStr">
         <is>
           <t>Header, data rows and Totals row are all rgb(249,250,251) (pale blue-grey), not white.</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="F62" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Inspect the row background colour.</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G62" s="4" t="inlineStr">
         <is>
           <t>Rows are white (with no alternating shading).</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr">
+      <c r="H62" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — row background colour; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="I62" s="4" t="inlineStr">
         <is>
           <t>SV-8970 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J24" s="4" t="inlineStr">
+      <c r="J62" s="4" t="inlineStr">
         <is>
           <t>Yes (exactly)</t>
         </is>
       </c>
-      <c r="K24" s="4" t="inlineStr">
+      <c r="K62" s="4" t="inlineStr">
         <is>
           <t>C30519 (https://shopview.testrail.io/index.php?/cases/view/30519)</t>
         </is>
       </c>
-      <c r="L24" s="4" t="inlineStr">
+      <c r="L62" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>18</t>
         </is>
       </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
+      <c r="B63" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D63" s="4" t="inlineStr">
         <is>
           <t>Numeric column headers/cells left-aligned</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E63" s="4" t="inlineStr">
         <is>
           <t>Days Open and Last Activity column headers are left-aligned (expected right); the Days Open data cell is also left-aligned. Broader than the ticket named.</t>
         </is>
       </c>
-      <c r="F25" s="4" t="inlineStr">
+      <c r="F63" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Check the alignment of the Days Open and Last Activity column headers and the Days Open data cells.</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G63" s="4" t="inlineStr">
         <is>
           <t>Numeric/right-hand columns (Days Open, Last Activity) are right-aligned.</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H63" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — column alignment; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I25" s="4" t="inlineStr">
+      <c r="I63" s="4" t="inlineStr">
         <is>
           <t>SV-8987 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J25" s="4" t="inlineStr">
+      <c r="J63" s="4" t="inlineStr">
         <is>
           <t>Yes (broader than the ticket)</t>
         </is>
       </c>
-      <c r="K25" s="4" t="inlineStr">
+      <c r="K63" s="4" t="inlineStr">
         <is>
           <t>C30466 (https://shopview.testrail.io/index.php?/cases/view/30466)</t>
         </is>
       </c>
-      <c r="L25" s="4" t="inlineStr">
+      <c r="L63" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>19</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D64" s="4" t="inlineStr">
         <is>
           <t>Estimates summary figure not muted</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E64" s="4" t="inlineStr">
         <is>
           <t>The Estimates summary figure is rgb(54,65,82) — identical to the others — so it is not toned down/muted.</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F64" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Compare the colour of the Estimates summary figure to the Completed and Not-Started figures.</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G64" s="4" t="inlineStr">
         <is>
           <t>The Estimates summary figure is toned down / muted relative to the others.</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — Estimates summary styling; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I26" s="4" t="inlineStr">
+      <c r="I64" s="4" t="inlineStr">
         <is>
           <t>SV-8988 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J26" s="4" t="inlineStr">
+      <c r="J64" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K26" s="4" t="inlineStr">
+      <c r="K64" s="4" t="inlineStr">
         <is>
           <t>C30491 (https://shopview.testrail.io/index.php?/cases/view/30491)</t>
         </is>
       </c>
-      <c r="L26" s="4" t="inlineStr">
+      <c r="L64" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="4" t="inlineStr">
         <is>
           <t>20</t>
         </is>
       </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D65" s="4" t="inlineStr">
         <is>
           <t>Labor Delta shows two decimals</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E65" s="4" t="inlineStr">
         <is>
           <t>Labor Delta shows two decimals (+3.00, +2.20); expected one decimal. Sign is correct.</t>
         </is>
       </c>
-      <c r="F27" s="4" t="inlineStr">
+      <c r="F65" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Read a Labor Delta value.</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="G65" s="4" t="inlineStr">
         <is>
           <t>Labor Delta shows one decimal (e.g. +3.0).</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H65" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — Labor Delta formatting; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I27" s="4" t="inlineStr">
+      <c r="I65" s="4" t="inlineStr">
         <is>
           <t>SV-8989 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J27" s="4" t="inlineStr">
+      <c r="J65" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K27" s="4" t="inlineStr">
+      <c r="K65" s="4" t="inlineStr">
         <is>
           <t>C30481 (https://shopview.testrail.io/index.php?/cases/view/30481)</t>
         </is>
       </c>
-      <c r="L27" s="4" t="inlineStr">
+      <c r="L65" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="4" t="inlineStr">
         <is>
           <t>21</t>
         </is>
       </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C66" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D66" s="4" t="inlineStr">
         <is>
           <t>Customer filter offers Clear before any selection</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E66" s="4" t="inlineStr">
         <is>
           <t>The Customer filter shows "Clear all" before anything is selected.</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="F66" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Open the Customer filter without selecting anything.
 3. Look for a Clear action.</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G66" s="4" t="inlineStr">
         <is>
           <t>No Clear action until at least one selection is made; then it is labelled "Clear".</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
+      <c r="H66" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — filter Clear behaviour; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I28" s="4" t="inlineStr">
+      <c r="I66" s="4" t="inlineStr">
         <is>
           <t>SV-8969 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J28" s="4" t="inlineStr">
+      <c r="J66" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K28" s="4" t="inlineStr">
+      <c r="K66" s="4" t="inlineStr">
         <is>
           <t>C30499 (https://shopview.testrail.io/index.php?/cases/view/30499)</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L66" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="4" t="inlineStr">
         <is>
           <t>22</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="B67" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D67" s="4" t="inlineStr">
         <is>
           <t>Filter change fires a server request</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E67" s="4" t="inlineStr">
         <is>
           <t>Changing a filter (e.g. Advisor) fires one server request (server-side recompute); figures are correct either way.</t>
         </is>
       </c>
-      <c r="F29" s="4" t="inlineStr">
+      <c r="F67" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Open dev tools Network.
@@ -1958,382 +2221,382 @@
 4. Watch for a server request.</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G67" s="4" t="inlineStr">
         <is>
           <t>The filter narrows the results on-screen with no server request.</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H67" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — client-side filter narrowing; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="I67" s="4" t="inlineStr">
         <is>
           <t>SV-8968 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
+      <c r="J67" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K29" s="4" t="inlineStr">
+      <c r="K67" s="4" t="inlineStr">
         <is>
           <t>C30505 (https://shopview.testrail.io/index.php?/cases/view/30505), C30498 (https://shopview.testrail.io/index.php?/cases/view/30498)</t>
         </is>
       </c>
-      <c r="L29" s="4" t="inlineStr">
+      <c r="L67" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="4" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>23</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C68" s="4" t="inlineStr">
         <is>
           <t>Inventory Value</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D68" s="4" t="inlineStr">
         <is>
           <t>Totals row reads "Totals" not "Total"</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E68" s="4" t="inlineStr">
         <is>
           <t>The Totals row's first cell reads "Totals"; the spec asks for "Total".</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="F68" s="4" t="inlineStr">
         <is>
           <t>1. Open Inventory Value.
 2. Read the first cell of the Totals row.</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G68" s="4" t="inlineStr">
         <is>
           <t>The Totals row's first cell reads "Total".</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>IV report specification v10 S4-R1; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I30" s="4" t="inlineStr">
+      <c r="I68" s="4" t="inlineStr">
         <is>
           <t>SV-8926 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
+      <c r="J68" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K30" s="4" t="inlineStr">
+      <c r="K68" s="4" t="inlineStr">
         <is>
           <t>C30556 (https://shopview.testrail.io/index.php?/cases/view/30556)</t>
         </is>
       </c>
-      <c r="L30" s="4" t="inlineStr">
+      <c r="L68" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="4" t="inlineStr">
         <is>
           <t>24</t>
         </is>
       </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
+      <c r="B69" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
         <is>
           <t>Inventory Value</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D69" s="4" t="inlineStr">
         <is>
           <t>Empty-state wording differs from spec</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E69" s="4" t="inlineStr">
         <is>
           <t>The empty-state message reads "No inventory value to show for this selection." — not the spec's standard wording.</t>
         </is>
       </c>
-      <c r="F31" s="4" t="inlineStr">
+      <c r="F69" s="4" t="inlineStr">
         <is>
           <t>1. Open Inventory Value.
 2. Apply a selection that returns no rows.
 3. Read the empty-state message.</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G69" s="4" t="inlineStr">
         <is>
           <t>The empty-state shows the spec's standard wording: "Empty bays, endless possibilities. Get Going!".</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H69" s="4" t="inlineStr">
         <is>
           <t>IV report specification v10 — standard empty-state wording; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I31" s="4" t="inlineStr">
+      <c r="I69" s="4" t="inlineStr">
         <is>
           <t>SV-8930 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J31" s="4" t="inlineStr">
+      <c r="J69" s="4" t="inlineStr">
         <is>
           <t>Yes (different wording)</t>
         </is>
       </c>
-      <c r="K31" s="4" t="inlineStr">
+      <c r="K69" s="4" t="inlineStr">
         <is>
           <t>C30539 (https://shopview.testrail.io/index.php?/cases/view/30539)</t>
         </is>
       </c>
-      <c r="L31" s="4" t="inlineStr">
+      <c r="L69" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="4" t="inlineStr">
         <is>
           <t>25</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C70" s="4" t="inlineStr">
         <is>
           <t>Inventory Value</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D70" s="4" t="inlineStr">
         <is>
           <t>First visit opens All locations</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E70" s="4" t="inlineStr">
         <is>
           <t>On first visit (fresh browser context) the report opens on "All locations", not the active location.</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="F70" s="4" t="inlineStr">
         <is>
           <t>1. Open Inventory Value in a fresh browser context.
 2. Check the Location default.</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G70" s="4" t="inlineStr">
         <is>
           <t>First visit opens on the user's active location.</t>
         </is>
       </c>
-      <c r="H32" s="4" t="inlineStr">
+      <c r="H70" s="4" t="inlineStr">
         <is>
           <t>IV report specification v10 S1-R3 / S7-R2; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="I70" s="4" t="inlineStr">
         <is>
           <t>SV-8931 (OBSOLETE)</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
+      <c r="J70" s="4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="K32" s="4" t="inlineStr">
+      <c r="K70" s="4" t="inlineStr">
         <is>
           <t>C30536 (https://shopview.testrail.io/index.php?/cases/view/30536), C30574 (https://shopview.testrail.io/index.php?/cases/view/30574)</t>
         </is>
       </c>
-      <c r="L32" s="4" t="inlineStr">
+      <c r="L70" s="4" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>26</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="B71" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
         <is>
           <t>Technician Utilization</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D71" s="4" t="inlineStr">
         <is>
           <t>Empty export shows an error toast instead of silent no-op</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E71" s="4" t="inlineStr">
         <is>
           <t>Exporting with all technicians cleared shows an "Empty export / Export didn't yield any results" error toast, not the spec's silent no-op. Differs from BOTH the spec and the old SV-8948 symptom.</t>
         </is>
       </c>
-      <c r="F33" s="4" t="inlineStr">
+      <c r="F71" s="4" t="inlineStr">
         <is>
           <t>1. Open Technician Utilization.
 2. Deselect all technicians.
 3. Trigger an export.</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G71" s="4" t="inlineStr">
         <is>
           <t>A silent no-op — no file is produced and no message is shown.</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H71" s="4" t="inlineStr">
         <is>
           <t>TU report specification v9 S7-N1 (silent no-op); epic SV-8582.</t>
         </is>
       </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="I71" s="4" t="inlineStr">
         <is>
           <t>NO TICKET (new deviation)</t>
         </is>
       </c>
-      <c r="J33" s="4" t="inlineStr">
+      <c r="J71" s="4" t="inlineStr">
         <is>
           <t>Yes (new deviation)</t>
         </is>
       </c>
-      <c r="K33" s="4" t="inlineStr">
+      <c r="K71" s="4" t="inlineStr">
         <is>
           <t>C30440 (https://shopview.testrail.io/index.php?/cases/view/30440)</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L71" s="4" t="inlineStr">
         <is>
           <t>FILE-NEW</t>
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+    <row r="72">
+      <c r="A72" s="4" t="inlineStr">
         <is>
           <t>27</t>
         </is>
       </c>
-      <c r="B34" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C34" s="4" t="inlineStr">
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C72" s="4" t="inlineStr">
         <is>
           <t>Sales By Representative / Inventory Value</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D72" s="4" t="inlineStr">
         <is>
           <t>CSV money now plain numbers (appears fixed)</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E72" s="4" t="inlineStr">
         <is>
           <t>CSV money is now written as plain numbers, not "$…" text; IV column order is also correct (Total Cost last).</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="F72" s="4" t="inlineStr">
         <is>
           <t>1. Open Sales By Representative (then Inventory Value).
 2. Export CSV.
 3. Open the file and check the money columns (and IV column order).</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G72" s="4" t="inlineStr">
         <is>
           <t>CSV money is plain numbers; IV Total Cost is the last column.</t>
         </is>
       </c>
-      <c r="H34" s="4" t="inlineStr">
+      <c r="H72" s="4" t="inlineStr">
         <is>
           <t>SBR / IV report specifications — CSV money format + IV column order; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I34" s="4" t="inlineStr">
+      <c r="I72" s="4" t="inlineStr">
         <is>
           <t>SV-8823 (OPEN — TESTING QA)</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr">
+      <c r="J72" s="4" t="inlineStr">
         <is>
           <t>No — appears FIXED on v3.8</t>
         </is>
       </c>
-      <c r="K34" s="4" t="inlineStr">
+      <c r="K72" s="4" t="inlineStr">
         <is>
           <t>C30287 (https://shopview.testrail.io/index.php?/cases/view/30287), C30589 (https://shopview.testrail.io/index.php?/cases/view/30589)</t>
         </is>
       </c>
-      <c r="L34" s="4" t="inlineStr">
+      <c r="L72" s="4" t="inlineStr">
         <is>
           <t>CLOSE-AS-FIXED (first verify the CSV honours column-selection-in-export — IV sub-claim not tested; C30588 keeps an SV-8823 note)</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="73">
+      <c r="A73" s="4" t="inlineStr">
         <is>
           <t>28</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="B73" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D73" s="4" t="inlineStr">
         <is>
           <t>✅ RESOLVED 2026-08-19 — PO question: WIP tab-placement spec self-contradiction</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>The spec carried BOTH placement models: S2-R4 ("appears once, in one tab") vs the SV-9027 line-state Key Decision ("appears in each matching tab"). RESOLVED by Chris Ward 2026-08-19 — he tidied the LIVE Confluence spec so Story 3 and S2-R4 now describe the line-state model (new S3-R5, S3-R6). Our cases already follow line-state (his 2026-08-18 answer B), so they now agree with the tidied spec; the divergence note can be retired. Still owed: pull the live page (local baseline v22 is behind).</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
+      <c r="E73" s="4" t="inlineStr">
+        <is>
+          <t>The spec carried BOTH placement models: S2-R4 ("appears once, in one tab") vs the SV-9027 line-state Key Decision ("appears in each matching tab"). **RESOLVED by Chris Ward 2026-08-19** — he tidied the LIVE Confluence spec so Story 3 and S2-R4 now describe the line-state model (new S3-R5, S3-R6). Our cases already follow line-state (his 2026-08-18 answer B), so they now agree with the tidied spec; the divergence note can be retired. Still owed: pull the live page (local baseline v22 is behind).</t>
+        </is>
+      </c>
+      <c r="F73" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Find a work order with lines in more than one state.
@@ -2341,492 +2604,485 @@
 (Note: no such WO exists in current data — needs seeding.)</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G73" s="4" t="inlineStr">
         <is>
           <t>Per the current documents (now consistent): a work order appears in each matching tab by line state (line-state model).</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H73" s="4" t="inlineStr">
         <is>
           <t>WIP report specification — live Confluence (line-state model, new S3-R5/S3-R6); Chris Ward ruling 2026-08-19.</t>
         </is>
       </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="I73" s="4" t="inlineStr">
         <is>
           <t>N/A (document conflict — RESOLVED by PO)</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
+      <c r="J73" s="4" t="inlineStr">
         <is>
           <t>Not established (no multi-state WO in data)</t>
         </is>
       </c>
-      <c r="K35" s="4" t="inlineStr">
+      <c r="K73" s="4" t="inlineStr">
         <is>
           <t>C30456 (https://shopview.testrail.io/index.php?/cases/view/30456), C30458 (https://shopview.testrail.io/index.php?/cases/view/30458), C43979 (https://shopview.testrail.io/index.php?/cases/view/43979)</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L73" s="4" t="inlineStr">
         <is>
           <t>RESOLVED (Chris Ward 2026-08-19 tidied the live spec to line-state; pull live page — register RS-WIP-6)</t>
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>29</t>
         </is>
       </c>
-      <c r="B36" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C36" s="4" t="inlineStr">
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C74" s="4" t="inlineStr">
         <is>
           <t>Sales By Customer / Sales By Representative</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D74" s="4" t="inlineStr">
         <is>
           <t>PO question: invoice number — link or plain text?</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E74" s="4" t="inlineStr">
         <is>
           <t>The build renders the invoice number as a plain-text span (no href), but the spec states BOTH: S9-N2 (link to access-denied) and S9-R1a (plain-text, no link).</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="F74" s="4" t="inlineStr">
         <is>
           <t>1. Open Sales By Customer (and Sales By Representative).
 2. Look at an invoice number cell — is it a link or plain text?</t>
         </is>
       </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="G74" s="4" t="inlineStr">
         <is>
           <t>Per the intended (to-be-confirmed) document: whichever of link / plain-text Chris Ward confirms.</t>
         </is>
       </c>
-      <c r="H36" s="4" t="inlineStr">
+      <c r="H74" s="4" t="inlineStr">
         <is>
           <t>SBC / SBR report specifications — conflict between S9-N2 and S9-R1a.</t>
         </is>
       </c>
-      <c r="I36" s="4" t="inlineStr">
+      <c r="I74" s="4" t="inlineStr">
         <is>
           <t>N/A (document conflict — not a defect)</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
+      <c r="J74" s="4" t="inlineStr">
         <is>
           <t>N/A (build shows plain text; conflict unresolved)</t>
         </is>
       </c>
-      <c r="K36" s="4" t="inlineStr">
+      <c r="K74" s="4" t="inlineStr">
         <is>
           <t>C30100 (https://shopview.testrail.io/index.php?/cases/view/30100), C43558 (https://shopview.testrail.io/index.php?/cases/view/43558), C30138 (https://shopview.testrail.io/index.php?/cases/view/30138)</t>
         </is>
       </c>
-      <c r="L36" s="4" t="inlineStr">
+      <c r="L74" s="4" t="inlineStr">
         <is>
           <t>PO-QUESTION (chase Chris Ward for the intended behaviour)</t>
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+    <row r="75">
+      <c r="A75" s="4" t="inlineStr">
         <is>
           <t>30</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="B75" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
         <is>
           <t>Parts Velocity</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D75" s="4" t="inlineStr">
         <is>
           <t>PO question: Location column position</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E75" s="4" t="inlineStr">
         <is>
           <t>SV-8938 says the Location column should be leftmost (before Type), but the spec says two different things (S3-R10 access-gated/toggleable vs S2-R12 scope-tied), and the 20 picker columns don't list Location. The column sits 6th on screen and in CSV.</t>
         </is>
       </c>
-      <c r="F37" s="4" t="inlineStr">
+      <c r="F75" s="4" t="inlineStr">
         <is>
           <t>1. Sign in as a multi-location user.
 2. Open Parts Velocity.
 3. Note the Location column position on screen and in the CSV export.</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G75" s="4" t="inlineStr">
         <is>
           <t>Per the intended (to-be-confirmed) document: the position/toggle behaviour Chris Ward confirms.</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H75" s="4" t="inlineStr">
         <is>
           <t>PV report specification — conflict between S3-R10 and S2-R12; contested ticket SV-8938.</t>
         </is>
       </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="I75" s="4" t="inlineStr">
         <is>
           <t>SV-8938 (contested)</t>
         </is>
       </c>
-      <c r="J37" s="4" t="inlineStr">
+      <c r="J75" s="4" t="inlineStr">
         <is>
           <t>Column sits 6th (on screen + CSV); "leftmost" not confirmed</t>
         </is>
       </c>
-      <c r="K37" s="4" t="inlineStr">
+      <c r="K75" s="4" t="inlineStr">
         <is>
           <t>C38914 (https://shopview.testrail.io/index.php?/cases/view/38914), C30352 (https://shopview.testrail.io/index.php?/cases/view/30352)</t>
         </is>
       </c>
-      <c r="L37" s="4" t="inlineStr">
+      <c r="L75" s="4" t="inlineStr">
         <is>
           <t>PO-QUESTION (get Chris Ward's answer before reopening/refiling SV-8938)</t>
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="4" t="inlineStr">
         <is>
           <t>31</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C76" s="4" t="inlineStr">
         <is>
           <t>Parts Velocity</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D76" s="4" t="inlineStr">
         <is>
           <t>PDF export fails (SV-8818)</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E76" s="4" t="inlineStr">
         <is>
           <t>PDF export returns HTTP 500 on a medium view while CSV works; over-cap views are correctly refused with the standard message.</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="F76" s="4" t="inlineStr">
         <is>
           <t>1. Open Parts Velocity.
 2. Load a medium-sized view.
 3. Export PDF.</t>
         </is>
       </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="G76" s="4" t="inlineStr">
         <is>
           <t>PDF export returns a downloadable file (HTTP 200).</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H76" s="4" t="inlineStr">
         <is>
           <t>PV report specification — PDF export requirement; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="I76" s="4" t="inlineStr">
         <is>
           <t>SV-8818 (OPEN — TESTING QA)</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
+      <c r="J76" s="4" t="inlineStr">
         <is>
           <t>Yes (PDF 500)</t>
         </is>
       </c>
-      <c r="K38" s="4" t="inlineStr">
+      <c r="K76" s="4" t="inlineStr">
         <is>
           <t>C38885 (https://shopview.testrail.io/index.php?/cases/view/38885), C43547 (https://shopview.testrail.io/index.php?/cases/view/43547)</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="L76" s="4" t="inlineStr">
         <is>
           <t>KEEP-EXPECT-FAIL</t>
         </is>
       </c>
     </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="B77" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
         <is>
           <t>Inventory Value</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D77" s="4" t="inlineStr">
         <is>
           <t>PDF export fails on large view (SV-8818)</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E77" s="4" t="inlineStr">
         <is>
           <t>PDF export times out / returns 500 on the large IV view (5,703 rows); small filtered views work (HTTP 200).</t>
         </is>
       </c>
-      <c r="F39" s="4" t="inlineStr">
+      <c r="F77" s="4" t="inlineStr">
         <is>
           <t>1. Open Inventory Value.
 2. Load the large (all-locations) view.
 3. Export PDF.</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G77" s="4" t="inlineStr">
         <is>
           <t>PDF export returns a downloadable file (HTTP 200).</t>
         </is>
       </c>
-      <c r="H39" s="4" t="inlineStr">
+      <c r="H77" s="4" t="inlineStr">
         <is>
           <t>IV report specification v10 — PDF export requirement; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="I77" s="4" t="inlineStr">
         <is>
           <t>SV-8818 (OPEN — TESTING QA)</t>
         </is>
       </c>
-      <c r="J39" s="4" t="inlineStr">
+      <c r="J77" s="4" t="inlineStr">
         <is>
           <t>Yes (PDF 500/timeout on large view)</t>
         </is>
       </c>
-      <c r="K39" s="4" t="inlineStr">
+      <c r="K77" s="4" t="inlineStr">
         <is>
           <t>C30587 (https://shopview.testrail.io/index.php?/cases/view/30587), C30590 (https://shopview.testrail.io/index.php?/cases/view/30590), C30591 (https://shopview.testrail.io/index.php?/cases/view/30591), C30593 (https://shopview.testrail.io/index.php?/cases/view/30593), C30595 (https://shopview.testrail.io/index.php?/cases/view/30595), C43548 (https://shopview.testrail.io/index.php?/cases/view/43548)</t>
         </is>
       </c>
-      <c r="L39" s="4" t="inlineStr">
+      <c r="L77" s="4" t="inlineStr">
         <is>
           <t>KEEP-EXPECT-FAIL</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>33</t>
         </is>
       </c>
-      <c r="B40" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C40" s="4" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>Sales By Representative</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>Over-cap Expanded PDF / API row-cap (SV-8818)</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E78" s="4" t="inlineStr">
         <is>
           <t>The &gt; row-cap Expanded-PDF / API state is not reachable at 88 invoices; base exports return 200. Kept EXPECT-FAIL pending a seedable over-cap state.</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="F78" s="4" t="inlineStr">
         <is>
           <t>1. Open Sales By Representative.
 2. Build a view that exceeds the row cap (not reachable at 88 invoices — needs seeding).
 3. Export the Expanded PDF.</t>
         </is>
       </c>
-      <c r="G40" s="4" t="inlineStr">
+      <c r="G78" s="4" t="inlineStr">
         <is>
           <t>Over-cap export is refused with the standard row-cap message.</t>
         </is>
       </c>
-      <c r="H40" s="4" t="inlineStr">
+      <c r="H78" s="4" t="inlineStr">
         <is>
           <t>SBR report specification — export row-cap; epic SV-8582.</t>
         </is>
       </c>
-      <c r="I40" s="4" t="inlineStr">
+      <c r="I78" s="4" t="inlineStr">
         <is>
           <t>SV-8818 (OPEN — TESTING QA)</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
+      <c r="J78" s="4" t="inlineStr">
         <is>
           <t>Not reachable at 88 invoices (base exports 200)</t>
         </is>
       </c>
-      <c r="K40" s="4" t="inlineStr">
+      <c r="K78" s="4" t="inlineStr">
         <is>
           <t>C30290 (https://shopview.testrail.io/index.php?/cases/view/30290), C30320 (https://shopview.testrail.io/index.php?/cases/view/30320)</t>
         </is>
       </c>
-      <c r="L40" s="4" t="inlineStr">
+      <c r="L78" s="4" t="inlineStr">
         <is>
           <t>KEEP-EXPECT-FAIL</t>
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>34</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>Schedule</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>Sidebar - Work Order Filters</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t>Priority filter group missing from the sidebar Filters panel</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E79" s="4" t="inlineStr">
         <is>
           <t>The sidebar Filters popup contains only Assignment (Unassigned/Assigned) and Status; there is no Priority group (High/Medium/Low). Confirmed by reading the full popup and a body-wide search.</t>
         </is>
       </c>
-      <c r="F41" s="4" t="inlineStr">
+      <c r="F79" s="4" t="inlineStr">
         <is>
           <t>1. Open Schedule.
 2. Click the sidebar Filters button.
 3. Look for a Priority group with High / Medium / Low options.</t>
         </is>
       </c>
-      <c r="G41" s="4" t="inlineStr">
+      <c r="G79" s="4" t="inlineStr">
         <is>
           <t>The Filters panel offers three groups: Assignment, Status, and Priority (High, Medium, Low).</t>
         </is>
       </c>
-      <c r="H41" s="4" t="inlineStr">
+      <c r="H79" s="4" t="inlineStr">
         <is>
           <t>Schedule specification v30 §5.1 / story SV-8687; epic SV-8685.</t>
         </is>
       </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="I79" s="4" t="inlineStr">
         <is>
           <t>NO TICKET (feature not found — Rule 69 deferred)</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr">
+      <c r="J79" s="4" t="inlineStr">
         <is>
           <t>Yes (Priority group absent on v3.8-bd246fd)</t>
         </is>
       </c>
-      <c r="K41" s="4" t="inlineStr">
+      <c r="K79" s="4" t="inlineStr">
         <is>
           <t>C29945 (https://shopview.testrail.io/index.php?/cases/view/29945)</t>
         </is>
       </c>
-      <c r="L41" s="4" t="inlineStr">
+      <c r="L79" s="4" t="inlineStr">
         <is>
           <t>DEFERRED (feature not found — confirm with Branko whether Priority filtering is in V1; re-check when it ships)</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>35</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
-        <is>
-          <t>Report Suite</t>
-        </is>
-      </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>Report Suite</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>Work In Progress</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D80" s="4" t="inlineStr">
         <is>
           <t>✅ RESOLVED 2026-08-19 — WIP aging is per job (FINAL); shared Days Open on a two-row job is correct</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>Chris Ward's 2nd message ruled aging is per job, and *"that's final"*. Days Open is whole days since the work order's date; a two-row job (status tab + Estimates) shows the same number on both rows — *"the money splits by line state, the clock doesn't"* — and that shared number is CORRECT behaviour, not a bug. The stray per-line-aging line is gone from the spec as of page v24, so nothing conflicts. A separate Quote Age column is future work — SV-9372 (Parth, not started); nothing to test — do NOT file the shared Days Open value as a defect in the meantime.</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="E80" s="4" t="inlineStr">
+        <is>
+          <t>Chris Ward's 2nd message ruled aging is **per job, and *"that's final"***. Days Open is whole days since the work order's date; a two-row job (status tab + Estimates) shows the **same** number on both rows — *"the money splits by line state, the clock doesn't"* — and that shared number is **CORRECT behaviour, not a bug**. The stray per-line-aging line is **gone from the spec as of page v24**, so nothing conflicts. **A separate Quote Age column is future work — SV-9372 (Parth, not started); nothing to test — do NOT file the shared Days Open value as a defect in the meantime.**</t>
+        </is>
+      </c>
+      <c r="F80" s="4" t="inlineStr">
         <is>
           <t>1. Open Work In Progress.
 2. Read the Days Open value for a work order that has both approved and unapproved lines (and appears on two tabs).
 3. Confirm it counts whole days since the work order's date (not per line), and that both rows show the same number.</t>
         </is>
       </c>
-      <c r="G42" s="4" t="inlineStr">
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>Days Open = whole days since the work order's date (S4-R12), per job; both rows of a two-row job show the same number (correct, not a defect). Per-line aging is NOT built — do not test for it. A future Quote Age column (SV-9372) is not yet built — nothing to test.</t>
         </is>
       </c>
-      <c r="H42" s="4" t="inlineStr">
+      <c r="H80" s="4" t="inlineStr">
         <is>
           <t>WIP report specification S4-R12 (per-line line removed as of page v24); Chris Ward 2nd ruling 2026-08-19.</t>
         </is>
       </c>
-      <c r="I42" s="4" t="inlineStr">
+      <c r="I80" s="4" t="inlineStr">
         <is>
           <t>N/A (RESOLVED by PO — per job, final)</t>
         </is>
       </c>
-      <c r="J42" s="4" t="inlineStr">
+      <c r="J80" s="4" t="inlineStr">
         <is>
           <t>Whole-job Days Open builds correctly; shared value on a two-row job is correct</t>
         </is>
       </c>
-      <c r="K42" s="4" t="inlineStr">
+      <c r="K80" s="4" t="inlineStr">
         <is>
           <t>C30472 (https://shopview.testrail.io/index.php?/cases/view/30472)</t>
         </is>
       </c>
-      <c r="L42" s="4" t="inlineStr">
+      <c r="L80" s="4" t="inlineStr">
         <is>
           <t>RESOLVED (Chris Ward 2026-08-19 — aging per job, final; do NOT file the shared Days Open value as a defect; SV-9372 Quote Age is future — register RS-WIP-4 cleared, RS-WIP-7 opened)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A5:L5"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="A4:L4"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2840,7 +3096,7 @@
   <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2854,7 +3110,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Schedule batches B (66 cases) and C (68 cases) are PENDING — their defect verdicts cannot be produced until fresh staging cookies land. This file covers Report Suite (all 6 reports) + Schedule batch A only.</t>
+          <t>| 35 | Report Suite | Work In Progress | ✅ RESOLVED 2026-08-19 — WIP aging is per job (FINAL); shared Days Open on a two-row job is correct | Chris Ward's 2nd message ruled aging is per job, and *"that's final"*. Days Open is whole days since the work order's date; a two-row job (status tab + Estimates) shows the same number on both rows — *"the money splits by line state, the clock doesn't"* — and that shared number is CORRECT behaviour, not a bug. The stray per-line-aging line is gone from the spec as of page v24, so nothing conflicts. A separate Quote Age column is future work — SV-9372 (Parth, not started); nothing to test — do NOT file the shared Days Open value as a defect in the meantime. | 1. Open Work In Progress.&lt;br&gt;2. Read the Days Open value for a work order that has both approved and unapproved lines (and appears on two tabs).&lt;br&gt;3. Confirm it counts whole days since the work order's date (not per line), and that both rows show the same number. | Days Open = whole days since the work order's date (S4-R12), per job; both rows of a two-row job show the same number (correct, not a defect). Per-line aging is NOT built — do not test for it. A future Quote Age column (SV-9372) is not yet built — nothing to test. | WIP report specification S4-R12 (per-line line removed as of page v24); Chris Ward 2nd ruling 2026-08-19. | N/A (RESOLVED by PO — per job, final) | Whole-job Days Open builds correctly; shared value on a two-row job is correct | C30472 (https://shopview.testrail.io/index.php?/cases/view/30472) | RESOLVED (Chris Ward 2026-08-19 — aging per job, final; do NOT file the shared Days Open value as a defect; SV-9372 Quote Age is future — register RS-WIP-4 cleared, RS-WIP-7 opened) |</t>
         </is>
       </c>
     </row>
@@ -2866,19 +3122,19 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>Report Suite</t>
         </is>
@@ -2888,7 +3144,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>Schedule</t>
         </is>
@@ -2898,13 +3154,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="n">
-        <v>35</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>**TOTAL**</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>**35**</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -2915,19 +3173,19 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Count</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>REOPEN</t>
         </is>
@@ -2937,7 +3195,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>PO-QUESTION</t>
         </is>
@@ -2947,7 +3205,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>RESOLVED (PO answer 2026-08-19)</t>
         </is>
@@ -2957,7 +3215,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>KEEP-EXPECT-FAIL</t>
         </is>
@@ -2967,7 +3225,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>FILE-NEW</t>
         </is>
@@ -2977,7 +3235,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>CLOSE-AS-FIXED</t>
         </is>
@@ -2987,7 +3245,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>DEFERRED</t>
         </is>
@@ -2997,20 +3255,18 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B19" s="9" t="n">
-        <v>35</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>**TOTAL**</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>**35**</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>